<commit_message>
Fix h-08 span: ReAssure Forever is clause 4.2.17, not 4.2.16 (Return+)
Caught while pulling the restoration trigger text for the reference-answer survey.
The h-08 table is the ReAssure Forever restoration worked example, but the span
had clause 4.2.16 - which is Return+, a premium-return benefit on the same page.
4.2.16 resolved (it is on p12), so nothing errored: a resolving-but-wrong clause
id, the exact silent mislabel this project guards against, one benefit clause
away from the right one. Corrected to 4.2.17 (ReAssure Forever) and the divergence
recorded in the row.

The six table_formula rows stay prepared, not started; v1.jsonl unchanged at 24.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/golden/v1.xlsx
+++ b/data/golden/v1.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>4.2.16|</t>
+          <t>4.2.17|</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr"/>
@@ -1159,7 +1159,7 @@
       <c r="M12" s="3" t="n"/>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>TABLE_FORMULA, STITCHED worked-example grid across nivabupa-rise p12-13 (ReAssure Forever restoration, clause 4.2.16). Same 9-column structure as h-07 but the sibling product's forever-restoration variant, Base Sum Insured 10 Lakh. Paired deliberately with h-07: the two restoration mechanisms look identical in the grid and differ in the trigger rule, so a system that stitches one correctly can still answer the other wrong. Same 10-Lakh-only caveat.</t>
+          <t>TABLE_FORMULA, STITCHED worked-example grid across nivabupa-rise p12-13 (ReAssure Forever restoration, clause 4.2.17 (NOT 4.2.16, which is Return+, a premium-return benefit - a resolving-but-wrong clause caught before import)). Same 9-column structure as h-07 but the sibling product's forever-restoration variant, Base Sum Insured 10 Lakh. Paired deliberately with h-07: the two restoration mechanisms look identical in the grid and differ in the trigger rule, so a system that stitches one correctly can still answer the other wrong. Same 10-Lakh-only caveat.</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">

</xml_diff>